<commit_message>
hh apc and additional costs data 2025 processed
</commit_message>
<xml_diff>
--- a/data/hh/original_data/apc_hal_2025.xlsx
+++ b/data/hh/original_data/apc_hal_2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\annrym\Desktop\STRAGISK FINANSIERIN\Open APC sweden 2025\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/2021m30/R/repos/openapc-se/data/hh/original_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{071D2B87-556C-4E70-9C00-86A56C63CB72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6EFA4DB-54F3-DD49-89F8-164CB7110FEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="76620" yWindow="1220" windowWidth="35840" windowHeight="21120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="article data" sheetId="1" r:id="rId1"/>
@@ -698,23 +698,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AB29"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.625" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.625" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="36.625" style="2" customWidth="1"/>
+    <col min="1" max="1" width="10.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.1640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="36.6640625" style="2" customWidth="1"/>
     <col min="5" max="5" width="10" style="2" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="37" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="38.625" style="2" customWidth="1"/>
-    <col min="8" max="8" width="5.125" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.625" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.875" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="3.375" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="38.6640625" style="2" customWidth="1"/>
+    <col min="8" max="8" width="5.1640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.83203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="3.33203125" style="2" bestFit="1" customWidth="1"/>
     <col min="12" max="16384" width="11" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="1" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -766,7 +766,7 @@
       <c r="AA1"/>
       <c r="AB1"/>
     </row>
-    <row r="2" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>54</v>
       </c>
@@ -812,7 +812,7 @@
       <c r="AA2"/>
       <c r="AB2"/>
     </row>
-    <row r="3" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>54</v>
       </c>
@@ -858,7 +858,7 @@
       <c r="AA3"/>
       <c r="AB3"/>
     </row>
-    <row r="4" spans="1:28" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" ht="19" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>54</v>
       </c>
@@ -904,7 +904,7 @@
       <c r="AA4"/>
       <c r="AB4"/>
     </row>
-    <row r="5" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>54</v>
       </c>
@@ -950,7 +950,7 @@
       <c r="AA5"/>
       <c r="AB5"/>
     </row>
-    <row r="6" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>54</v>
       </c>
@@ -996,7 +996,7 @@
       <c r="AA6"/>
       <c r="AB6"/>
     </row>
-    <row r="7" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>54</v>
       </c>
@@ -1042,7 +1042,7 @@
       <c r="AA7"/>
       <c r="AB7"/>
     </row>
-    <row r="8" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>54</v>
       </c>
@@ -1088,7 +1088,7 @@
       <c r="AA8"/>
       <c r="AB8"/>
     </row>
-    <row r="9" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>54</v>
       </c>
@@ -1134,7 +1134,7 @@
       <c r="AA9"/>
       <c r="AB9"/>
     </row>
-    <row r="10" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>54</v>
       </c>
@@ -1180,7 +1180,7 @@
       <c r="AA10"/>
       <c r="AB10"/>
     </row>
-    <row r="11" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>54</v>
       </c>
@@ -1226,7 +1226,7 @@
       <c r="AA11"/>
       <c r="AB11"/>
     </row>
-    <row r="12" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>54</v>
       </c>
@@ -1272,7 +1272,7 @@
       <c r="AA12"/>
       <c r="AB12"/>
     </row>
-    <row r="13" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>54</v>
       </c>
@@ -1318,7 +1318,7 @@
       <c r="AA13"/>
       <c r="AB13"/>
     </row>
-    <row r="14" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>54</v>
       </c>
@@ -1364,7 +1364,7 @@
       <c r="AA14"/>
       <c r="AB14"/>
     </row>
-    <row r="15" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>54</v>
       </c>
@@ -1410,7 +1410,7 @@
       <c r="AA15"/>
       <c r="AB15"/>
     </row>
-    <row r="16" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A16" s="13" t="s">
         <v>54</v>
       </c>
@@ -1456,7 +1456,7 @@
       <c r="AA16"/>
       <c r="AB16"/>
     </row>
-    <row r="17" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>54</v>
       </c>
@@ -1502,7 +1502,7 @@
       <c r="AA17"/>
       <c r="AB17"/>
     </row>
-    <row r="18" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A18"/>
       <c r="B18"/>
       <c r="C18"/>
@@ -1532,7 +1532,7 @@
       <c r="AA18"/>
       <c r="AB18"/>
     </row>
-    <row r="19" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A19" s="13" t="s">
         <v>67</v>
       </c>
@@ -1564,7 +1564,7 @@
       <c r="AA19"/>
       <c r="AB19"/>
     </row>
-    <row r="20" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A20"/>
       <c r="B20"/>
       <c r="C20"/>
@@ -1594,7 +1594,7 @@
       <c r="AA20"/>
       <c r="AB20"/>
     </row>
-    <row r="21" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A21"/>
       <c r="B21"/>
       <c r="C21" s="13"/>
@@ -1624,7 +1624,7 @@
       <c r="AA21"/>
       <c r="AB21"/>
     </row>
-    <row r="22" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A22"/>
       <c r="B22"/>
       <c r="C22"/>
@@ -1654,7 +1654,7 @@
       <c r="AA22"/>
       <c r="AB22"/>
     </row>
-    <row r="23" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A23"/>
       <c r="B23"/>
       <c r="C23"/>
@@ -1684,7 +1684,7 @@
       <c r="AA23"/>
       <c r="AB23"/>
     </row>
-    <row r="24" spans="1:28" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:28" s="4" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A24"/>
       <c r="B24"/>
       <c r="C24"/>
@@ -1714,7 +1714,7 @@
       <c r="AA24"/>
       <c r="AB24"/>
     </row>
-    <row r="25" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A25"/>
       <c r="B25"/>
       <c r="C25"/>
@@ -1744,7 +1744,7 @@
       <c r="AA25"/>
       <c r="AB25"/>
     </row>
-    <row r="26" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A26"/>
       <c r="B26"/>
       <c r="C26"/>
@@ -1774,7 +1774,7 @@
       <c r="AA26"/>
       <c r="AB26"/>
     </row>
-    <row r="27" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A27"/>
       <c r="B27"/>
       <c r="C27"/>
@@ -1804,7 +1804,7 @@
       <c r="AA27"/>
       <c r="AB27"/>
     </row>
-    <row r="28" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A28"/>
       <c r="B28"/>
       <c r="C28"/>
@@ -1834,7 +1834,7 @@
       <c r="AA28"/>
       <c r="AB28"/>
     </row>
-    <row r="29" spans="1:28" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:28" x14ac:dyDescent="0.2">
       <c r="E29" s="8"/>
     </row>
   </sheetData>
@@ -1863,21 +1863,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4E9D608-332C-6B41-B918-E0AD75CD6855}">
   <dimension ref="A1:X4"/>
-  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="26.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="7.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="7.875" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="10.875" style="1"/>
+    <col min="9" max="10" width="7.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -1909,7 +1909,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>41</v>
       </c>
@@ -1917,7 +1917,7 @@
         <v>3170.82</v>
       </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.2">
       <c r="S4" s="5"/>
       <c r="T4" s="5"/>
       <c r="U4" s="5"/>

</xml_diff>